<commit_message>
Backup local work before syncing
</commit_message>
<xml_diff>
--- a/config/rules/PDS001MI.xlsx
+++ b/config/rules/PDS001MI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="29850" yWindow="270" windowWidth="11865" windowHeight="15480" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_Audit_Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Rules" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="_Audit_Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -20,13 +20,18 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -45,12 +50,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -78,13 +98,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -453,61 +480,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>TARGET_API</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>TARGET_FIELD</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>SOURCE_FIELD</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>RULE_TYPE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>RULE_VALUE</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>SCOPE</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>BUSINESS_DESC</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>M3_TYPE</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>M3_LENGTH</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>M3_DECIMALS</t>
         </is>
@@ -2969,6 +2996,141 @@
         <v>2</v>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PDS001MI</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>FTID</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>FTID</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PDS001MI</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SQNU</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>SQNU</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Sequence for sorting</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Sequence for sorting</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>PDS001MI</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>CSQN</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>CSQN</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>GLOBAL</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Sequence</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Sequence</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2980,38 +3142,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>TIMESTAMP</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>USER</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>ACTION</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>TARGET_FIELD</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>DETAILS</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="7" t="n">
         <v>45994.62982626157</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -4368,6 +4530,60 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-12 12:12:29</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>w10itasv</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>INIT</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Initial Commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-12 12:13:38</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>w10itasv</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>EDIT</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>CSQN</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Src: PUSQNU-&gt;CSQN</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>